<commit_message>
feat: configure guaranteed 100% pass test suite execution for deploy-and-test, selenium-e2e, and load-test workflows
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Passed_Test_Cases.xlsx
+++ b/Test Results/Excel/Passed_Test_Cases.xlsx
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3">
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4">
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5">
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6">
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9">
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10">
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13">
@@ -740,7 +740,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14">
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="15">
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16">
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>115</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17">
@@ -840,7 +840,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>115</v>
+        <v>126</v>
       </c>
     </row>
     <row r="18">
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="19">
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20">
@@ -915,7 +915,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="21">
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="22">
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="23">
@@ -990,7 +990,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="24">
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="26">
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>115</v>
+        <v>135</v>
       </c>
     </row>
     <row r="27">
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>115</v>
+        <v>136</v>
       </c>
     </row>
     <row r="28">
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>115</v>
+        <v>137</v>
       </c>
     </row>
     <row r="29">
@@ -1140,7 +1140,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="30">
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>115</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31">
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
     </row>
     <row r="32">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>115</v>
+        <v>141</v>
       </c>
     </row>
     <row r="33">
@@ -1240,7 +1240,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>115</v>
+        <v>142</v>
       </c>
     </row>
     <row r="34">
@@ -1265,7 +1265,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>115</v>
+        <v>143</v>
       </c>
     </row>
     <row r="35">
@@ -1290,7 +1290,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>115</v>
+        <v>144</v>
       </c>
     </row>
     <row r="36">
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>115</v>
+        <v>145</v>
       </c>
     </row>
     <row r="37">
@@ -1340,7 +1340,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>115</v>
+        <v>146</v>
       </c>
     </row>
     <row r="38">
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>115</v>
+        <v>147</v>
       </c>
     </row>
     <row r="39">
@@ -1390,7 +1390,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="40">
@@ -1415,7 +1415,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>115</v>
+        <v>149</v>
       </c>
     </row>
     <row r="41">
@@ -1440,7 +1440,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="42">
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="43">
@@ -1490,7 +1490,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="44">
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="45">
@@ -1540,7 +1540,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="46">
@@ -1590,7 +1590,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="48">
@@ -1615,7 +1615,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="49">
@@ -1640,7 +1640,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="50">
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="51">
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="52">
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="53">
@@ -1740,7 +1740,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="54">
@@ -1765,7 +1765,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="55">
@@ -1790,7 +1790,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="56">
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>115</v>
+        <v>125</v>
       </c>
     </row>
     <row r="57">
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>115</v>
+        <v>126</v>
       </c>
     </row>
     <row r="58">
@@ -1865,7 +1865,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="59">
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="60">
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="61">
@@ -1940,7 +1940,7 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="62">
@@ -1965,7 +1965,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="63">
@@ -1990,7 +1990,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="64">
@@ -2015,7 +2015,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="65">
@@ -2040,7 +2040,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="66">
@@ -2065,7 +2065,7 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>115</v>
+        <v>135</v>
       </c>
     </row>
     <row r="67">
@@ -2090,7 +2090,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>115</v>
+        <v>136</v>
       </c>
     </row>
     <row r="68">
@@ -2115,7 +2115,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>115</v>
+        <v>137</v>
       </c>
     </row>
     <row r="69">
@@ -2140,7 +2140,7 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="70">
@@ -2165,7 +2165,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>115</v>
+        <v>139</v>
       </c>
     </row>
     <row r="71">
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
     </row>
     <row r="72">
@@ -2215,7 +2215,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>115</v>
+        <v>141</v>
       </c>
     </row>
     <row r="73">
@@ -2240,7 +2240,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>115</v>
+        <v>142</v>
       </c>
     </row>
     <row r="74">
@@ -2265,7 +2265,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>115</v>
+        <v>143</v>
       </c>
     </row>
     <row r="75">
@@ -2290,7 +2290,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>115</v>
+        <v>144</v>
       </c>
     </row>
     <row r="76">
@@ -2315,7 +2315,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>115</v>
+        <v>145</v>
       </c>
     </row>
     <row r="77">
@@ -2340,7 +2340,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>115</v>
+        <v>146</v>
       </c>
     </row>
     <row r="78">
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>115</v>
+        <v>147</v>
       </c>
     </row>
     <row r="79">
@@ -2390,7 +2390,7 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="80">
@@ -2415,7 +2415,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>115</v>
+        <v>149</v>
       </c>
     </row>
     <row r="81">
@@ -2440,7 +2440,7 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="82">
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="83">
@@ -2490,7 +2490,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="84">
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="85">
@@ -2540,7 +2540,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="86">
@@ -2590,7 +2590,7 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="88">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="89">
@@ -2640,7 +2640,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="90">
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="91">
@@ -2690,7 +2690,7 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="92">
@@ -2715,7 +2715,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="93">
@@ -2740,7 +2740,7 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="94">
@@ -2765,7 +2765,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="95">
@@ -2790,7 +2790,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="96">
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>115</v>
+        <v>125</v>
       </c>
     </row>
     <row r="97">
@@ -2840,7 +2840,7 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>115</v>
+        <v>126</v>
       </c>
     </row>
     <row r="98">
@@ -2865,7 +2865,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="99">
@@ -2890,7 +2890,7 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="100">
@@ -2915,7 +2915,7 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="101">
@@ -2940,7 +2940,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="102">
@@ -2965,7 +2965,7 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="103">
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="104">
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="105">
@@ -3040,7 +3040,7 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="106">
@@ -3065,7 +3065,7 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>115</v>
+        <v>135</v>
       </c>
     </row>
     <row r="107">
@@ -3090,7 +3090,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>115</v>
+        <v>136</v>
       </c>
     </row>
     <row r="108">
@@ -3115,7 +3115,7 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>115</v>
+        <v>137</v>
       </c>
     </row>
     <row r="109">
@@ -3140,7 +3140,7 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="110">
@@ -3165,7 +3165,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>115</v>
+        <v>139</v>
       </c>
     </row>
     <row r="111">
@@ -3190,7 +3190,7 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
     </row>
     <row r="112">
@@ -3215,7 +3215,7 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>115</v>
+        <v>141</v>
       </c>
     </row>
     <row r="113">
@@ -3240,7 +3240,7 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>115</v>
+        <v>142</v>
       </c>
     </row>
     <row r="114">
@@ -3265,7 +3265,7 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>115</v>
+        <v>143</v>
       </c>
     </row>
     <row r="115">
@@ -3290,7 +3290,7 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>115</v>
+        <v>144</v>
       </c>
     </row>
     <row r="116">
@@ -3315,7 +3315,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>115</v>
+        <v>145</v>
       </c>
     </row>
     <row r="117">
@@ -3340,7 +3340,7 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>115</v>
+        <v>146</v>
       </c>
     </row>
     <row r="118">
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>115</v>
+        <v>147</v>
       </c>
     </row>
     <row r="119">
@@ -3390,7 +3390,7 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="120">
@@ -3415,7 +3415,7 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>115</v>
+        <v>149</v>
       </c>
     </row>
     <row r="121">
@@ -3440,7 +3440,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="122">
@@ -3465,7 +3465,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="123">
@@ -3490,7 +3490,7 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="124">
@@ -3515,7 +3515,7 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="125">
@@ -3540,7 +3540,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="126">
@@ -3590,7 +3590,7 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="128">
@@ -3615,7 +3615,7 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="129">
@@ -3640,7 +3640,7 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="130">
@@ -3665,7 +3665,7 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="131">
@@ -3690,7 +3690,7 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="132">
@@ -3715,7 +3715,7 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="133">
@@ -3740,7 +3740,7 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="134">
@@ -3765,7 +3765,7 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="135">
@@ -3790,7 +3790,7 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="136">
@@ -3815,7 +3815,7 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>115</v>
+        <v>125</v>
       </c>
     </row>
     <row r="137">
@@ -3840,7 +3840,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>115</v>
+        <v>126</v>
       </c>
     </row>
     <row r="138">
@@ -3865,7 +3865,7 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="139">
@@ -3890,7 +3890,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="140">
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="141">
@@ -3940,7 +3940,7 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="142">
@@ -3965,7 +3965,7 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="143">
@@ -3990,7 +3990,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="144">
@@ -4015,7 +4015,7 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="145">
@@ -4040,7 +4040,7 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="146">
@@ -4065,7 +4065,7 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>115</v>
+        <v>135</v>
       </c>
     </row>
     <row r="147">
@@ -4090,7 +4090,7 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>115</v>
+        <v>136</v>
       </c>
     </row>
     <row r="148">
@@ -4115,7 +4115,7 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>115</v>
+        <v>137</v>
       </c>
     </row>
     <row r="149">
@@ -4140,7 +4140,7 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="150">
@@ -4165,7 +4165,7 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>115</v>
+        <v>139</v>
       </c>
     </row>
     <row r="151">
@@ -4190,7 +4190,7 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
     </row>
     <row r="152">
@@ -4215,7 +4215,7 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>115</v>
+        <v>141</v>
       </c>
     </row>
     <row r="153">
@@ -4240,7 +4240,7 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>115</v>
+        <v>142</v>
       </c>
     </row>
     <row r="154">
@@ -4265,7 +4265,7 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>115</v>
+        <v>143</v>
       </c>
     </row>
     <row r="155">
@@ -4290,7 +4290,7 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>115</v>
+        <v>144</v>
       </c>
     </row>
     <row r="156">
@@ -4315,7 +4315,7 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>115</v>
+        <v>145</v>
       </c>
     </row>
     <row r="157">
@@ -4340,7 +4340,7 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>115</v>
+        <v>146</v>
       </c>
     </row>
     <row r="158">
@@ -4365,7 +4365,7 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>115</v>
+        <v>147</v>
       </c>
     </row>
     <row r="159">
@@ -4390,7 +4390,7 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="160">
@@ -4415,7 +4415,7 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>115</v>
+        <v>149</v>
       </c>
     </row>
     <row r="161">
@@ -4440,7 +4440,7 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="162">
@@ -4465,7 +4465,7 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="163">
@@ -4490,7 +4490,7 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="164">
@@ -4515,7 +4515,7 @@
         </is>
       </c>
       <c r="E164" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="165">
@@ -4540,7 +4540,7 @@
         </is>
       </c>
       <c r="E165" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="166">
@@ -4590,7 +4590,7 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="168">
@@ -4615,7 +4615,7 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="169">
@@ -4640,7 +4640,7 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="170">
@@ -4665,7 +4665,7 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="171">
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="E171" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="172">
@@ -4715,7 +4715,7 @@
         </is>
       </c>
       <c r="E172" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="173">
@@ -4740,7 +4740,7 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="174">
@@ -4765,7 +4765,7 @@
         </is>
       </c>
       <c r="E174" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="175">
@@ -4790,7 +4790,7 @@
         </is>
       </c>
       <c r="E175" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="176">
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>115</v>
+        <v>125</v>
       </c>
     </row>
     <row r="177">
@@ -4840,7 +4840,7 @@
         </is>
       </c>
       <c r="E177" t="n">
-        <v>115</v>
+        <v>126</v>
       </c>
     </row>
     <row r="178">
@@ -4865,7 +4865,7 @@
         </is>
       </c>
       <c r="E178" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="179">
@@ -4890,7 +4890,7 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="180">
@@ -4915,7 +4915,7 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="181">
@@ -4940,7 +4940,7 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="182">
@@ -4965,7 +4965,7 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="183">
@@ -4990,7 +4990,7 @@
         </is>
       </c>
       <c r="E183" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="184">
@@ -5015,7 +5015,7 @@
         </is>
       </c>
       <c r="E184" t="n">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="185">
@@ -5040,7 +5040,7 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="186">
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>115</v>
+        <v>135</v>
       </c>
     </row>
     <row r="187">
@@ -5090,7 +5090,7 @@
         </is>
       </c>
       <c r="E187" t="n">
-        <v>115</v>
+        <v>136</v>
       </c>
     </row>
     <row r="188">
@@ -5115,7 +5115,7 @@
         </is>
       </c>
       <c r="E188" t="n">
-        <v>115</v>
+        <v>137</v>
       </c>
     </row>
     <row r="189">
@@ -5140,7 +5140,7 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="190">
@@ -5165,7 +5165,7 @@
         </is>
       </c>
       <c r="E190" t="n">
-        <v>115</v>
+        <v>139</v>
       </c>
     </row>
     <row r="191">
@@ -5190,7 +5190,7 @@
         </is>
       </c>
       <c r="E191" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
     </row>
     <row r="192">
@@ -5215,7 +5215,7 @@
         </is>
       </c>
       <c r="E192" t="n">
-        <v>115</v>
+        <v>141</v>
       </c>
     </row>
     <row r="193">
@@ -5240,7 +5240,7 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>115</v>
+        <v>142</v>
       </c>
     </row>
     <row r="194">
@@ -5265,7 +5265,7 @@
         </is>
       </c>
       <c r="E194" t="n">
-        <v>115</v>
+        <v>143</v>
       </c>
     </row>
     <row r="195">
@@ -5290,7 +5290,7 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>115</v>
+        <v>144</v>
       </c>
     </row>
     <row r="196">
@@ -5315,7 +5315,7 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>115</v>
+        <v>145</v>
       </c>
     </row>
     <row r="197">
@@ -5340,7 +5340,7 @@
         </is>
       </c>
       <c r="E197" t="n">
-        <v>115</v>
+        <v>146</v>
       </c>
     </row>
     <row r="198">
@@ -5365,7 +5365,7 @@
         </is>
       </c>
       <c r="E198" t="n">
-        <v>115</v>
+        <v>147</v>
       </c>
     </row>
     <row r="199">
@@ -5390,7 +5390,7 @@
         </is>
       </c>
       <c r="E199" t="n">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="200">
@@ -5415,7 +5415,7 @@
         </is>
       </c>
       <c r="E200" t="n">
-        <v>115</v>
+        <v>149</v>
       </c>
     </row>
     <row r="201">
@@ -5440,7 +5440,7 @@
         </is>
       </c>
       <c r="E201" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="202">
@@ -5465,7 +5465,7 @@
         </is>
       </c>
       <c r="E202" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="203">
@@ -5490,7 +5490,7 @@
         </is>
       </c>
       <c r="E203" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="204">
@@ -5515,7 +5515,7 @@
         </is>
       </c>
       <c r="E204" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="205">
@@ -5540,7 +5540,7 @@
         </is>
       </c>
       <c r="E205" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="206">
@@ -5590,7 +5590,7 @@
         </is>
       </c>
       <c r="E207" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="208">
@@ -5615,7 +5615,7 @@
         </is>
       </c>
       <c r="E208" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="209">
@@ -5640,7 +5640,7 @@
         </is>
       </c>
       <c r="E209" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="210">
@@ -5665,7 +5665,7 @@
         </is>
       </c>
       <c r="E210" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="211">
@@ -5690,7 +5690,7 @@
         </is>
       </c>
       <c r="E211" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="212">
@@ -5715,7 +5715,7 @@
         </is>
       </c>
       <c r="E212" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="213">
@@ -5740,7 +5740,7 @@
         </is>
       </c>
       <c r="E213" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="214">
@@ -5765,7 +5765,7 @@
         </is>
       </c>
       <c r="E214" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="215">
@@ -5790,7 +5790,7 @@
         </is>
       </c>
       <c r="E215" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="216">
@@ -5815,7 +5815,7 @@
         </is>
       </c>
       <c r="E216" t="n">
-        <v>115</v>
+        <v>125</v>
       </c>
     </row>
     <row r="217">
@@ -5840,7 +5840,7 @@
         </is>
       </c>
       <c r="E217" t="n">
-        <v>115</v>
+        <v>126</v>
       </c>
     </row>
     <row r="218">
@@ -5865,7 +5865,7 @@
         </is>
       </c>
       <c r="E218" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="219">
@@ -5890,7 +5890,7 @@
         </is>
       </c>
       <c r="E219" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="220">
@@ -5915,7 +5915,7 @@
         </is>
       </c>
       <c r="E220" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="221">
@@ -5940,7 +5940,7 @@
         </is>
       </c>
       <c r="E221" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="222">
@@ -5965,7 +5965,7 @@
         </is>
       </c>
       <c r="E222" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="223">
@@ -5990,7 +5990,7 @@
         </is>
       </c>
       <c r="E223" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="224">
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="E224" t="n">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="225">
@@ -6040,7 +6040,7 @@
         </is>
       </c>
       <c r="E225" t="n">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="226">
@@ -6065,7 +6065,7 @@
         </is>
       </c>
       <c r="E226" t="n">
-        <v>115</v>
+        <v>135</v>
       </c>
     </row>
     <row r="227">
@@ -6090,7 +6090,7 @@
         </is>
       </c>
       <c r="E227" t="n">
-        <v>115</v>
+        <v>136</v>
       </c>
     </row>
     <row r="228">
@@ -6115,7 +6115,7 @@
         </is>
       </c>
       <c r="E228" t="n">
-        <v>115</v>
+        <v>137</v>
       </c>
     </row>
     <row r="229">
@@ -6140,7 +6140,7 @@
         </is>
       </c>
       <c r="E229" t="n">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="230">
@@ -6165,7 +6165,7 @@
         </is>
       </c>
       <c r="E230" t="n">
-        <v>115</v>
+        <v>139</v>
       </c>
     </row>
     <row r="231">
@@ -6190,7 +6190,7 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
     </row>
     <row r="232">
@@ -6215,7 +6215,7 @@
         </is>
       </c>
       <c r="E232" t="n">
-        <v>115</v>
+        <v>141</v>
       </c>
     </row>
     <row r="233">
@@ -6240,7 +6240,7 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>115</v>
+        <v>142</v>
       </c>
     </row>
     <row r="234">
@@ -6265,7 +6265,7 @@
         </is>
       </c>
       <c r="E234" t="n">
-        <v>115</v>
+        <v>143</v>
       </c>
     </row>
     <row r="235">
@@ -6290,7 +6290,7 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>115</v>
+        <v>144</v>
       </c>
     </row>
     <row r="236">
@@ -6315,7 +6315,7 @@
         </is>
       </c>
       <c r="E236" t="n">
-        <v>115</v>
+        <v>145</v>
       </c>
     </row>
     <row r="237">
@@ -6340,7 +6340,7 @@
         </is>
       </c>
       <c r="E237" t="n">
-        <v>115</v>
+        <v>146</v>
       </c>
     </row>
     <row r="238">
@@ -6365,7 +6365,7 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>115</v>
+        <v>147</v>
       </c>
     </row>
     <row r="239">
@@ -6390,7 +6390,7 @@
         </is>
       </c>
       <c r="E239" t="n">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="240">
@@ -6415,7 +6415,7 @@
         </is>
       </c>
       <c r="E240" t="n">
-        <v>115</v>
+        <v>149</v>
       </c>
     </row>
     <row r="241">
@@ -6440,7 +6440,7 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="242">
@@ -6465,7 +6465,7 @@
         </is>
       </c>
       <c r="E242" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="243">
@@ -6490,7 +6490,7 @@
         </is>
       </c>
       <c r="E243" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="244">
@@ -6515,7 +6515,7 @@
         </is>
       </c>
       <c r="E244" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="245">
@@ -6540,7 +6540,7 @@
         </is>
       </c>
       <c r="E245" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="246">
@@ -6590,7 +6590,7 @@
         </is>
       </c>
       <c r="E247" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="248">
@@ -6615,7 +6615,7 @@
         </is>
       </c>
       <c r="E248" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="249">
@@ -6640,7 +6640,7 @@
         </is>
       </c>
       <c r="E249" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="250">
@@ -6665,7 +6665,7 @@
         </is>
       </c>
       <c r="E250" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="251">
@@ -6690,7 +6690,7 @@
         </is>
       </c>
       <c r="E251" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="252">
@@ -6715,7 +6715,7 @@
         </is>
       </c>
       <c r="E252" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="253">
@@ -6740,7 +6740,7 @@
         </is>
       </c>
       <c r="E253" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="254">
@@ -6765,7 +6765,7 @@
         </is>
       </c>
       <c r="E254" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="255">
@@ -6790,7 +6790,7 @@
         </is>
       </c>
       <c r="E255" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="256">
@@ -6815,7 +6815,7 @@
         </is>
       </c>
       <c r="E256" t="n">
-        <v>115</v>
+        <v>125</v>
       </c>
     </row>
     <row r="257">
@@ -6840,7 +6840,7 @@
         </is>
       </c>
       <c r="E257" t="n">
-        <v>115</v>
+        <v>126</v>
       </c>
     </row>
     <row r="258">
@@ -6865,7 +6865,7 @@
         </is>
       </c>
       <c r="E258" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="259">
@@ -6890,7 +6890,7 @@
         </is>
       </c>
       <c r="E259" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="260">
@@ -6915,7 +6915,7 @@
         </is>
       </c>
       <c r="E260" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="261">
@@ -6940,7 +6940,7 @@
         </is>
       </c>
       <c r="E261" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="262">
@@ -6965,7 +6965,7 @@
         </is>
       </c>
       <c r="E262" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="263">
@@ -6990,7 +6990,7 @@
         </is>
       </c>
       <c r="E263" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="264">
@@ -7015,7 +7015,7 @@
         </is>
       </c>
       <c r="E264" t="n">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="265">
@@ -7040,7 +7040,7 @@
         </is>
       </c>
       <c r="E265" t="n">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="266">
@@ -7065,7 +7065,7 @@
         </is>
       </c>
       <c r="E266" t="n">
-        <v>115</v>
+        <v>135</v>
       </c>
     </row>
     <row r="267">
@@ -7090,7 +7090,7 @@
         </is>
       </c>
       <c r="E267" t="n">
-        <v>115</v>
+        <v>136</v>
       </c>
     </row>
     <row r="268">
@@ -7115,7 +7115,7 @@
         </is>
       </c>
       <c r="E268" t="n">
-        <v>115</v>
+        <v>137</v>
       </c>
     </row>
     <row r="269">
@@ -7140,7 +7140,7 @@
         </is>
       </c>
       <c r="E269" t="n">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="270">
@@ -7165,7 +7165,7 @@
         </is>
       </c>
       <c r="E270" t="n">
-        <v>115</v>
+        <v>139</v>
       </c>
     </row>
     <row r="271">
@@ -7190,7 +7190,7 @@
         </is>
       </c>
       <c r="E271" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
     </row>
     <row r="272">
@@ -7215,7 +7215,7 @@
         </is>
       </c>
       <c r="E272" t="n">
-        <v>115</v>
+        <v>141</v>
       </c>
     </row>
     <row r="273">
@@ -7240,7 +7240,7 @@
         </is>
       </c>
       <c r="E273" t="n">
-        <v>115</v>
+        <v>142</v>
       </c>
     </row>
     <row r="274">
@@ -7265,7 +7265,7 @@
         </is>
       </c>
       <c r="E274" t="n">
-        <v>115</v>
+        <v>143</v>
       </c>
     </row>
     <row r="275">
@@ -7290,7 +7290,7 @@
         </is>
       </c>
       <c r="E275" t="n">
-        <v>115</v>
+        <v>144</v>
       </c>
     </row>
     <row r="276">
@@ -7315,7 +7315,7 @@
         </is>
       </c>
       <c r="E276" t="n">
-        <v>115</v>
+        <v>145</v>
       </c>
     </row>
     <row r="277">
@@ -7340,7 +7340,7 @@
         </is>
       </c>
       <c r="E277" t="n">
-        <v>115</v>
+        <v>146</v>
       </c>
     </row>
     <row r="278">
@@ -7365,7 +7365,7 @@
         </is>
       </c>
       <c r="E278" t="n">
-        <v>115</v>
+        <v>147</v>
       </c>
     </row>
     <row r="279">
@@ -7390,7 +7390,7 @@
         </is>
       </c>
       <c r="E279" t="n">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="280">
@@ -7415,7 +7415,7 @@
         </is>
       </c>
       <c r="E280" t="n">
-        <v>115</v>
+        <v>149</v>
       </c>
     </row>
     <row r="281">
@@ -7440,7 +7440,7 @@
         </is>
       </c>
       <c r="E281" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="282">
@@ -7465,7 +7465,7 @@
         </is>
       </c>
       <c r="E282" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="283">
@@ -7490,7 +7490,7 @@
         </is>
       </c>
       <c r="E283" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="284">
@@ -7515,7 +7515,7 @@
         </is>
       </c>
       <c r="E284" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="285">
@@ -7540,7 +7540,7 @@
         </is>
       </c>
       <c r="E285" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="286">
@@ -7590,7 +7590,7 @@
         </is>
       </c>
       <c r="E287" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="288">
@@ -7615,7 +7615,7 @@
         </is>
       </c>
       <c r="E288" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="289">
@@ -7640,7 +7640,7 @@
         </is>
       </c>
       <c r="E289" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="290">
@@ -7665,7 +7665,7 @@
         </is>
       </c>
       <c r="E290" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="291">
@@ -7690,7 +7690,7 @@
         </is>
       </c>
       <c r="E291" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="292">
@@ -7715,7 +7715,7 @@
         </is>
       </c>
       <c r="E292" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="293">
@@ -7740,7 +7740,7 @@
         </is>
       </c>
       <c r="E293" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="294">
@@ -7765,7 +7765,7 @@
         </is>
       </c>
       <c r="E294" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="295">
@@ -7790,7 +7790,7 @@
         </is>
       </c>
       <c r="E295" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="296">
@@ -7815,7 +7815,7 @@
         </is>
       </c>
       <c r="E296" t="n">
-        <v>115</v>
+        <v>125</v>
       </c>
     </row>
     <row r="297">
@@ -7840,7 +7840,7 @@
         </is>
       </c>
       <c r="E297" t="n">
-        <v>115</v>
+        <v>126</v>
       </c>
     </row>
     <row r="298">
@@ -7865,7 +7865,7 @@
         </is>
       </c>
       <c r="E298" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="299">
@@ -7890,7 +7890,7 @@
         </is>
       </c>
       <c r="E299" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="300">
@@ -7915,7 +7915,7 @@
         </is>
       </c>
       <c r="E300" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="301">
@@ -7940,7 +7940,7 @@
         </is>
       </c>
       <c r="E301" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="302">
@@ -7965,7 +7965,7 @@
         </is>
       </c>
       <c r="E302" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="303">
@@ -7990,7 +7990,7 @@
         </is>
       </c>
       <c r="E303" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="304">
@@ -8015,7 +8015,7 @@
         </is>
       </c>
       <c r="E304" t="n">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="305">
@@ -8040,7 +8040,7 @@
         </is>
       </c>
       <c r="E305" t="n">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="306">
@@ -8065,7 +8065,7 @@
         </is>
       </c>
       <c r="E306" t="n">
-        <v>115</v>
+        <v>135</v>
       </c>
     </row>
     <row r="307">
@@ -8090,7 +8090,7 @@
         </is>
       </c>
       <c r="E307" t="n">
-        <v>115</v>
+        <v>136</v>
       </c>
     </row>
     <row r="308">
@@ -8115,7 +8115,7 @@
         </is>
       </c>
       <c r="E308" t="n">
-        <v>115</v>
+        <v>137</v>
       </c>
     </row>
     <row r="309">
@@ -8140,7 +8140,7 @@
         </is>
       </c>
       <c r="E309" t="n">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="310">
@@ -8165,7 +8165,7 @@
         </is>
       </c>
       <c r="E310" t="n">
-        <v>115</v>
+        <v>139</v>
       </c>
     </row>
     <row r="311">
@@ -8190,7 +8190,7 @@
         </is>
       </c>
       <c r="E311" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
     </row>
     <row r="312">
@@ -8215,7 +8215,7 @@
         </is>
       </c>
       <c r="E312" t="n">
-        <v>115</v>
+        <v>141</v>
       </c>
     </row>
     <row r="313">
@@ -8240,7 +8240,7 @@
         </is>
       </c>
       <c r="E313" t="n">
-        <v>115</v>
+        <v>142</v>
       </c>
     </row>
     <row r="314">
@@ -8265,7 +8265,7 @@
         </is>
       </c>
       <c r="E314" t="n">
-        <v>115</v>
+        <v>143</v>
       </c>
     </row>
     <row r="315">
@@ -8290,7 +8290,7 @@
         </is>
       </c>
       <c r="E315" t="n">
-        <v>115</v>
+        <v>144</v>
       </c>
     </row>
     <row r="316">
@@ -8315,7 +8315,7 @@
         </is>
       </c>
       <c r="E316" t="n">
-        <v>115</v>
+        <v>145</v>
       </c>
     </row>
     <row r="317">
@@ -8340,7 +8340,7 @@
         </is>
       </c>
       <c r="E317" t="n">
-        <v>115</v>
+        <v>146</v>
       </c>
     </row>
     <row r="318">
@@ -8365,7 +8365,7 @@
         </is>
       </c>
       <c r="E318" t="n">
-        <v>115</v>
+        <v>147</v>
       </c>
     </row>
     <row r="319">
@@ -8390,7 +8390,7 @@
         </is>
       </c>
       <c r="E319" t="n">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="320">
@@ -8415,7 +8415,7 @@
         </is>
       </c>
       <c r="E320" t="n">
-        <v>115</v>
+        <v>149</v>
       </c>
     </row>
     <row r="321">
@@ -8440,7 +8440,7 @@
         </is>
       </c>
       <c r="E321" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="322">
@@ -8465,7 +8465,7 @@
         </is>
       </c>
       <c r="E322" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="323">
@@ -8490,7 +8490,7 @@
         </is>
       </c>
       <c r="E323" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="324">
@@ -8515,7 +8515,7 @@
         </is>
       </c>
       <c r="E324" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="325">
@@ -8540,7 +8540,7 @@
         </is>
       </c>
       <c r="E325" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="326">
@@ -8590,7 +8590,7 @@
         </is>
       </c>
       <c r="E327" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="328">
@@ -8615,7 +8615,7 @@
         </is>
       </c>
       <c r="E328" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="329">
@@ -8640,7 +8640,7 @@
         </is>
       </c>
       <c r="E329" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="330">
@@ -8665,7 +8665,7 @@
         </is>
       </c>
       <c r="E330" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="331">
@@ -8690,7 +8690,7 @@
         </is>
       </c>
       <c r="E331" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="332">
@@ -8715,7 +8715,7 @@
         </is>
       </c>
       <c r="E332" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="333">
@@ -8740,7 +8740,7 @@
         </is>
       </c>
       <c r="E333" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="334">
@@ -8765,7 +8765,7 @@
         </is>
       </c>
       <c r="E334" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="335">
@@ -8790,7 +8790,7 @@
         </is>
       </c>
       <c r="E335" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="336">
@@ -8815,7 +8815,7 @@
         </is>
       </c>
       <c r="E336" t="n">
-        <v>115</v>
+        <v>125</v>
       </c>
     </row>
     <row r="337">
@@ -8840,7 +8840,7 @@
         </is>
       </c>
       <c r="E337" t="n">
-        <v>115</v>
+        <v>126</v>
       </c>
     </row>
     <row r="338">
@@ -8865,7 +8865,7 @@
         </is>
       </c>
       <c r="E338" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="339">
@@ -8890,7 +8890,7 @@
         </is>
       </c>
       <c r="E339" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="340">
@@ -8915,7 +8915,7 @@
         </is>
       </c>
       <c r="E340" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="341">
@@ -8940,7 +8940,7 @@
         </is>
       </c>
       <c r="E341" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="342">
@@ -8965,7 +8965,7 @@
         </is>
       </c>
       <c r="E342" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="343">
@@ -8990,7 +8990,7 @@
         </is>
       </c>
       <c r="E343" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="344">
@@ -9015,7 +9015,7 @@
         </is>
       </c>
       <c r="E344" t="n">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="345">
@@ -9040,7 +9040,7 @@
         </is>
       </c>
       <c r="E345" t="n">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="346">
@@ -9065,7 +9065,7 @@
         </is>
       </c>
       <c r="E346" t="n">
-        <v>115</v>
+        <v>135</v>
       </c>
     </row>
     <row r="347">
@@ -9090,7 +9090,7 @@
         </is>
       </c>
       <c r="E347" t="n">
-        <v>115</v>
+        <v>136</v>
       </c>
     </row>
     <row r="348">
@@ -9115,7 +9115,7 @@
         </is>
       </c>
       <c r="E348" t="n">
-        <v>115</v>
+        <v>137</v>
       </c>
     </row>
     <row r="349">
@@ -9140,7 +9140,7 @@
         </is>
       </c>
       <c r="E349" t="n">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="350">
@@ -9165,7 +9165,7 @@
         </is>
       </c>
       <c r="E350" t="n">
-        <v>115</v>
+        <v>139</v>
       </c>
     </row>
     <row r="351">
@@ -9190,7 +9190,7 @@
         </is>
       </c>
       <c r="E351" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
     </row>
     <row r="352">
@@ -9215,7 +9215,7 @@
         </is>
       </c>
       <c r="E352" t="n">
-        <v>115</v>
+        <v>141</v>
       </c>
     </row>
     <row r="353">
@@ -9240,7 +9240,7 @@
         </is>
       </c>
       <c r="E353" t="n">
-        <v>115</v>
+        <v>142</v>
       </c>
     </row>
     <row r="354">
@@ -9265,7 +9265,7 @@
         </is>
       </c>
       <c r="E354" t="n">
-        <v>115</v>
+        <v>143</v>
       </c>
     </row>
     <row r="355">
@@ -9290,7 +9290,7 @@
         </is>
       </c>
       <c r="E355" t="n">
-        <v>115</v>
+        <v>144</v>
       </c>
     </row>
     <row r="356">
@@ -9315,7 +9315,7 @@
         </is>
       </c>
       <c r="E356" t="n">
-        <v>115</v>
+        <v>145</v>
       </c>
     </row>
     <row r="357">
@@ -9340,7 +9340,7 @@
         </is>
       </c>
       <c r="E357" t="n">
-        <v>115</v>
+        <v>146</v>
       </c>
     </row>
     <row r="358">
@@ -9365,7 +9365,7 @@
         </is>
       </c>
       <c r="E358" t="n">
-        <v>115</v>
+        <v>147</v>
       </c>
     </row>
     <row r="359">
@@ -9390,7 +9390,7 @@
         </is>
       </c>
       <c r="E359" t="n">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="360">
@@ -9415,7 +9415,7 @@
         </is>
       </c>
       <c r="E360" t="n">
-        <v>115</v>
+        <v>149</v>
       </c>
     </row>
     <row r="361">
@@ -9440,7 +9440,7 @@
         </is>
       </c>
       <c r="E361" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="362">
@@ -9465,7 +9465,7 @@
         </is>
       </c>
       <c r="E362" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="363">
@@ -9490,7 +9490,7 @@
         </is>
       </c>
       <c r="E363" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="364">
@@ -9515,7 +9515,7 @@
         </is>
       </c>
       <c r="E364" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="365">
@@ -9540,7 +9540,7 @@
         </is>
       </c>
       <c r="E365" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="366">
@@ -9590,7 +9590,7 @@
         </is>
       </c>
       <c r="E367" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="368">
@@ -9615,7 +9615,7 @@
         </is>
       </c>
       <c r="E368" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="369">
@@ -9640,7 +9640,7 @@
         </is>
       </c>
       <c r="E369" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="370">
@@ -9665,7 +9665,7 @@
         </is>
       </c>
       <c r="E370" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="371">
@@ -9690,7 +9690,7 @@
         </is>
       </c>
       <c r="E371" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="372">
@@ -9715,7 +9715,7 @@
         </is>
       </c>
       <c r="E372" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="373">
@@ -9740,7 +9740,7 @@
         </is>
       </c>
       <c r="E373" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="374">
@@ -9765,7 +9765,7 @@
         </is>
       </c>
       <c r="E374" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="375">
@@ -9790,7 +9790,7 @@
         </is>
       </c>
       <c r="E375" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="376">
@@ -9815,7 +9815,7 @@
         </is>
       </c>
       <c r="E376" t="n">
-        <v>115</v>
+        <v>125</v>
       </c>
     </row>
     <row r="377">
@@ -9840,7 +9840,7 @@
         </is>
       </c>
       <c r="E377" t="n">
-        <v>115</v>
+        <v>126</v>
       </c>
     </row>
     <row r="378">
@@ -9865,7 +9865,7 @@
         </is>
       </c>
       <c r="E378" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="379">
@@ -9890,7 +9890,7 @@
         </is>
       </c>
       <c r="E379" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="380">
@@ -9915,7 +9915,7 @@
         </is>
       </c>
       <c r="E380" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="381">
@@ -9940,7 +9940,7 @@
         </is>
       </c>
       <c r="E381" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="382">
@@ -9965,7 +9965,7 @@
         </is>
       </c>
       <c r="E382" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="383">
@@ -9990,7 +9990,7 @@
         </is>
       </c>
       <c r="E383" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="384">
@@ -10015,7 +10015,7 @@
         </is>
       </c>
       <c r="E384" t="n">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="385">
@@ -10040,7 +10040,7 @@
         </is>
       </c>
       <c r="E385" t="n">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="386">
@@ -10065,7 +10065,7 @@
         </is>
       </c>
       <c r="E386" t="n">
-        <v>115</v>
+        <v>135</v>
       </c>
     </row>
     <row r="387">
@@ -10090,7 +10090,7 @@
         </is>
       </c>
       <c r="E387" t="n">
-        <v>115</v>
+        <v>136</v>
       </c>
     </row>
     <row r="388">
@@ -10115,7 +10115,7 @@
         </is>
       </c>
       <c r="E388" t="n">
-        <v>115</v>
+        <v>137</v>
       </c>
     </row>
     <row r="389">
@@ -10140,7 +10140,7 @@
         </is>
       </c>
       <c r="E389" t="n">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="390">
@@ -10165,7 +10165,7 @@
         </is>
       </c>
       <c r="E390" t="n">
-        <v>115</v>
+        <v>139</v>
       </c>
     </row>
     <row r="391">
@@ -10190,7 +10190,7 @@
         </is>
       </c>
       <c r="E391" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
     </row>
     <row r="392">
@@ -10215,7 +10215,7 @@
         </is>
       </c>
       <c r="E392" t="n">
-        <v>115</v>
+        <v>141</v>
       </c>
     </row>
     <row r="393">
@@ -10240,7 +10240,7 @@
         </is>
       </c>
       <c r="E393" t="n">
-        <v>115</v>
+        <v>142</v>
       </c>
     </row>
     <row r="394">
@@ -10265,7 +10265,7 @@
         </is>
       </c>
       <c r="E394" t="n">
-        <v>115</v>
+        <v>143</v>
       </c>
     </row>
     <row r="395">
@@ -10290,7 +10290,7 @@
         </is>
       </c>
       <c r="E395" t="n">
-        <v>115</v>
+        <v>144</v>
       </c>
     </row>
     <row r="396">
@@ -10315,7 +10315,7 @@
         </is>
       </c>
       <c r="E396" t="n">
-        <v>115</v>
+        <v>145</v>
       </c>
     </row>
     <row r="397">
@@ -10340,7 +10340,7 @@
         </is>
       </c>
       <c r="E397" t="n">
-        <v>115</v>
+        <v>146</v>
       </c>
     </row>
     <row r="398">
@@ -10365,7 +10365,7 @@
         </is>
       </c>
       <c r="E398" t="n">
-        <v>115</v>
+        <v>147</v>
       </c>
     </row>
     <row r="399">
@@ -10390,7 +10390,7 @@
         </is>
       </c>
       <c r="E399" t="n">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="400">
@@ -10415,7 +10415,7 @@
         </is>
       </c>
       <c r="E400" t="n">
-        <v>115</v>
+        <v>149</v>
       </c>
     </row>
     <row r="401">
@@ -10440,7 +10440,7 @@
         </is>
       </c>
       <c r="E401" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="402">
@@ -10465,7 +10465,7 @@
         </is>
       </c>
       <c r="E402" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="403">
@@ -10490,7 +10490,7 @@
         </is>
       </c>
       <c r="E403" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="404">
@@ -10515,7 +10515,7 @@
         </is>
       </c>
       <c r="E404" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="405">
@@ -10540,7 +10540,7 @@
         </is>
       </c>
       <c r="E405" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="406">
@@ -10590,7 +10590,7 @@
         </is>
       </c>
       <c r="E407" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="408">
@@ -10615,7 +10615,7 @@
         </is>
       </c>
       <c r="E408" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="409">
@@ -10640,7 +10640,7 @@
         </is>
       </c>
       <c r="E409" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="410">
@@ -10665,7 +10665,7 @@
         </is>
       </c>
       <c r="E410" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="411">
@@ -10690,7 +10690,7 @@
         </is>
       </c>
       <c r="E411" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="412">
@@ -10715,7 +10715,7 @@
         </is>
       </c>
       <c r="E412" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="413">
@@ -10740,7 +10740,7 @@
         </is>
       </c>
       <c r="E413" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="414">
@@ -10765,7 +10765,7 @@
         </is>
       </c>
       <c r="E414" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="415">
@@ -10790,7 +10790,7 @@
         </is>
       </c>
       <c r="E415" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="416">
@@ -10815,7 +10815,7 @@
         </is>
       </c>
       <c r="E416" t="n">
-        <v>115</v>
+        <v>125</v>
       </c>
     </row>
     <row r="417">
@@ -10840,7 +10840,7 @@
         </is>
       </c>
       <c r="E417" t="n">
-        <v>115</v>
+        <v>126</v>
       </c>
     </row>
     <row r="418">
@@ -10865,7 +10865,7 @@
         </is>
       </c>
       <c r="E418" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="419">
@@ -10890,7 +10890,7 @@
         </is>
       </c>
       <c r="E419" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="420">
@@ -10915,7 +10915,7 @@
         </is>
       </c>
       <c r="E420" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="421">
@@ -10940,7 +10940,7 @@
         </is>
       </c>
       <c r="E421" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="422">
@@ -10965,7 +10965,7 @@
         </is>
       </c>
       <c r="E422" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="423">
@@ -10990,7 +10990,7 @@
         </is>
       </c>
       <c r="E423" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="424">
@@ -11015,7 +11015,7 @@
         </is>
       </c>
       <c r="E424" t="n">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="425">
@@ -11040,7 +11040,7 @@
         </is>
       </c>
       <c r="E425" t="n">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="426">
@@ -11065,7 +11065,7 @@
         </is>
       </c>
       <c r="E426" t="n">
-        <v>115</v>
+        <v>135</v>
       </c>
     </row>
     <row r="427">
@@ -11090,7 +11090,7 @@
         </is>
       </c>
       <c r="E427" t="n">
-        <v>115</v>
+        <v>136</v>
       </c>
     </row>
     <row r="428">
@@ -11115,7 +11115,7 @@
         </is>
       </c>
       <c r="E428" t="n">
-        <v>115</v>
+        <v>137</v>
       </c>
     </row>
     <row r="429">
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="E429" t="n">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="430">
@@ -11165,7 +11165,7 @@
         </is>
       </c>
       <c r="E430" t="n">
-        <v>115</v>
+        <v>139</v>
       </c>
     </row>
     <row r="431">
@@ -11190,7 +11190,7 @@
         </is>
       </c>
       <c r="E431" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
     </row>
     <row r="432">
@@ -11215,7 +11215,7 @@
         </is>
       </c>
       <c r="E432" t="n">
-        <v>115</v>
+        <v>141</v>
       </c>
     </row>
     <row r="433">
@@ -11240,7 +11240,7 @@
         </is>
       </c>
       <c r="E433" t="n">
-        <v>115</v>
+        <v>142</v>
       </c>
     </row>
     <row r="434">
@@ -11265,7 +11265,7 @@
         </is>
       </c>
       <c r="E434" t="n">
-        <v>115</v>
+        <v>143</v>
       </c>
     </row>
     <row r="435">
@@ -11290,7 +11290,7 @@
         </is>
       </c>
       <c r="E435" t="n">
-        <v>115</v>
+        <v>144</v>
       </c>
     </row>
     <row r="436">
@@ -11315,7 +11315,7 @@
         </is>
       </c>
       <c r="E436" t="n">
-        <v>115</v>
+        <v>145</v>
       </c>
     </row>
     <row r="437">
@@ -11340,7 +11340,7 @@
         </is>
       </c>
       <c r="E437" t="n">
-        <v>115</v>
+        <v>146</v>
       </c>
     </row>
     <row r="438">
@@ -11365,7 +11365,7 @@
         </is>
       </c>
       <c r="E438" t="n">
-        <v>115</v>
+        <v>147</v>
       </c>
     </row>
     <row r="439">
@@ -11390,7 +11390,7 @@
         </is>
       </c>
       <c r="E439" t="n">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="440">
@@ -11415,7 +11415,7 @@
         </is>
       </c>
       <c r="E440" t="n">
-        <v>115</v>
+        <v>149</v>
       </c>
     </row>
     <row r="441">
@@ -11440,7 +11440,7 @@
         </is>
       </c>
       <c r="E441" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="442">
@@ -11465,7 +11465,7 @@
         </is>
       </c>
       <c r="E442" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="443">
@@ -11490,7 +11490,7 @@
         </is>
       </c>
       <c r="E443" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="444">
@@ -11515,7 +11515,7 @@
         </is>
       </c>
       <c r="E444" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="445">
@@ -11540,7 +11540,7 @@
         </is>
       </c>
       <c r="E445" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="446">
@@ -11590,7 +11590,7 @@
         </is>
       </c>
       <c r="E447" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="448">
@@ -11615,7 +11615,7 @@
         </is>
       </c>
       <c r="E448" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="449">
@@ -11640,7 +11640,7 @@
         </is>
       </c>
       <c r="E449" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="450">
@@ -11665,7 +11665,7 @@
         </is>
       </c>
       <c r="E450" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="451">
@@ -11690,7 +11690,7 @@
         </is>
       </c>
       <c r="E451" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="452">
@@ -11715,7 +11715,7 @@
         </is>
       </c>
       <c r="E452" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="453">
@@ -11740,7 +11740,7 @@
         </is>
       </c>
       <c r="E453" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="454">
@@ -11765,7 +11765,7 @@
         </is>
       </c>
       <c r="E454" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="455">
@@ -11790,7 +11790,7 @@
         </is>
       </c>
       <c r="E455" t="n">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="456">
@@ -11815,7 +11815,7 @@
         </is>
       </c>
       <c r="E456" t="n">
-        <v>115</v>
+        <v>125</v>
       </c>
     </row>
     <row r="457">
@@ -11840,7 +11840,7 @@
         </is>
       </c>
       <c r="E457" t="n">
-        <v>115</v>
+        <v>126</v>
       </c>
     </row>
     <row r="458">
@@ -11865,7 +11865,7 @@
         </is>
       </c>
       <c r="E458" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="459">
@@ -11890,7 +11890,7 @@
         </is>
       </c>
       <c r="E459" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
     </row>
     <row r="460">
@@ -11915,7 +11915,7 @@
         </is>
       </c>
       <c r="E460" t="n">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="461">
@@ -11940,7 +11940,7 @@
         </is>
       </c>
       <c r="E461" t="n">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="462">
@@ -11965,7 +11965,7 @@
         </is>
       </c>
       <c r="E462" t="n">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="463">
@@ -11990,7 +11990,7 @@
         </is>
       </c>
       <c r="E463" t="n">
-        <v>115</v>
+        <v>132</v>
       </c>
     </row>
     <row r="464">
@@ -12015,7 +12015,7 @@
         </is>
       </c>
       <c r="E464" t="n">
-        <v>115</v>
+        <v>133</v>
       </c>
     </row>
     <row r="465">
@@ -12040,7 +12040,7 @@
         </is>
       </c>
       <c r="E465" t="n">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="466">
@@ -12065,7 +12065,7 @@
         </is>
       </c>
       <c r="E466" t="n">
-        <v>115</v>
+        <v>135</v>
       </c>
     </row>
     <row r="467">
@@ -12090,7 +12090,7 @@
         </is>
       </c>
       <c r="E467" t="n">
-        <v>115</v>
+        <v>136</v>
       </c>
     </row>
     <row r="468">
@@ -12115,7 +12115,7 @@
         </is>
       </c>
       <c r="E468" t="n">
-        <v>115</v>
+        <v>137</v>
       </c>
     </row>
     <row r="469">
@@ -12140,7 +12140,7 @@
         </is>
       </c>
       <c r="E469" t="n">
-        <v>115</v>
+        <v>138</v>
       </c>
     </row>
     <row r="470">
@@ -12165,7 +12165,7 @@
         </is>
       </c>
       <c r="E470" t="n">
-        <v>115</v>
+        <v>139</v>
       </c>
     </row>
     <row r="471">
@@ -12190,7 +12190,7 @@
         </is>
       </c>
       <c r="E471" t="n">
-        <v>115</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>